<commit_message>
Cải thiện import trùng, tìm kiếm một phần và mẫu 2 người
- Thêm search_fill.py: tìm theo CCCD/họ tên/SĐT (nhập một phần)
- import_excel: xử lý TRUNG, ghi DaImport, kiểm tra SĐT 10 số
- Excel mẫu 2 người (TRẦN NGỌC DUNG + LE THI MAI) với sheet TimKiem/DaImport
- README: hướng dẫn trùng lặp và tra cứu

Co-authored-by: thaison20101 <thaison20101@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/kskdk-tthc-nhap-lieu/KSKDK_TTHC_mau_nhap.xlsx
+++ b/kskdk-tthc-nhap-lieu/KSKDK_TTHC_mau_nhap.xlsx
@@ -22,6 +22,8 @@
     <sheet name="DM_XaPhuong" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="DM_NgheNghiep" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="DM_NoiCongTac" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="TimKiem" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="DaImport" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -466,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -508,7 +510,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>2) Cột danh mục: gõ đúng Name hoặc Id như sheet DM_*</t>
@@ -516,7 +517,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>3) Ngày tháng: dd/MM/yyyy (ví dụ 29/07/2026)</t>
@@ -524,7 +524,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>4) Giới tính: Nam hoặc Nữ</t>
@@ -532,36 +531,40 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>5) Chạy: python3 import_excel.py --excel KSKDK_TTHC_mau_nhap.xlsx --user ... --password ...</t>
+          <t>5) Chạy import: python3 import_excel.py --excel KSKDK_TTHC_mau_nhap.xlsx --user ... --password ...</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>6) Thử trước: thêm --dry-run --limit 1</t>
+          <t>6) Tìm một phần: nhập CCCD/họ tên/SĐT ở sheet TimKiem → python3 search_fill.py --excel ...</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>7) Nếu người đã khám cùng ngày: TrangThai=TRUNG (không tạo bản ghi mới)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Lưu ý</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Web không có nút Import — script này gọi API FormToDatabaseInsert thay thế</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr">
+    <row r="11">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Không commit mật khẩu vào git</t>
         </is>
@@ -3033,13 +3036,686 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TÌM KIẾM (nhập một phần cũng được)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CCCD (đủ hoặc vài số cuối)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HoTen (một phần)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SDT (một phần)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NgaySinh</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Số kết quả</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HoTen (kết quả)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TRẦN NGỌC DUNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CCCD</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>087187000236</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SDT</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0989681925</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>NgaySinh</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>27/06/1987</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>MaBanGhi</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>904629</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TrangThai</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>THANH_CONG</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>GhiChu</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Đã import trước đó</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Chạy: python3 search_fill.py --excel KSKDK_TTHC_mau_nhap.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HoTen</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CCCD</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>SDT</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>MaBanGhi</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>TrangThai</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Nguon</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TRẦN NGỌC DUNG</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>087187000236</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0989681925</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>904629</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>THANH_CONG</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>DaImport:2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TRẦN NGỌC DUNG</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>087187000236</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0989681925</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>NhapLieu:3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>NgayKham</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>DoiTuong</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>DiaDiemKham</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>HinhThucChiTra</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>HinhThucKham</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>NguonKhac_GhiRo</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>CCCD</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>HoTen</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>NgaySinh</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>GioiTinh</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>DanToc</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>NhomMau</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>YeuToNhomMau</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>BHYT</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>SDT</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>NoiOHienTai</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>TinhThanh</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>XaPhuong</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>NgheNghiepId</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>NgheNghiep</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>NoiCongTac</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>XaPhuongCongTac</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>LyDoKham</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>MaBanGhi</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>TrangThai</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>GhiChu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Người lao động (theo pháp luật về an toàn, vệ sinh lao động)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Khám Lưu Động</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngân sách thành phố hỗ trợ </t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Khám Theo Hợp Đồng</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>087187000236</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>TRẦN NGỌC DUNG</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>27/06/1987</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0989681925</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>262/20 LẠC LONG QUÂN</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Thành Phố Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Phường Bình Thới</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>GIÁO VIÊN MẦM NON</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="X2" t="n">
+        <v>904629</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>THANH_CONG</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Đã import trước đó</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Người lao động (theo pháp luật về an toàn, vệ sinh lao động)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Khám Lưu Động</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngân sách thành phố hỗ trợ </t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Khám Theo Hợp Đồng</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>087187000236</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>TRẦN NGỌC DUNG</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>27/06/1987</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Kinh</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0989681925</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>262/20 LẠC LONG QUÂN</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Thành Phố Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Phường Bình Thới</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>GIÁO VIÊN MẦM NON</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 29/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Người lao động (theo pháp luật về an toàn, vệ sinh lao động)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Khám Lưu Động</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngân sách thành phố hỗ trợ </t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Khám Theo Hợp Đồng</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>079195031510</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>LE THI MAI</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>15/03/1995</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Kinh</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0989681920</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>45 Le Loi</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Thành Phố Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Phường Hiệp Bình</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>GIÁO VIÊN MẦM NON</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 29/07/2026</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:Z4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3065,6 +3741,9 @@
     <col width="18" customWidth="1" min="21" max="21"/>
     <col width="18" customWidth="1" min="22" max="22"/>
     <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -3183,6 +3862,21 @@
           <t>LyDoKham</t>
         </is>
       </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>MaBanGhi</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>TrangThai</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>GhiChu</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -3300,6 +3994,21 @@
           <t>Lý do khám sức khỏe</t>
         </is>
       </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>Script ghi — mã bản ghi trên web</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>THANH_CONG / TRUNG / LOI</t>
+        </is>
+      </c>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>Thông báo từ hệ thống</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3309,43 +4018,42 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sinh Viên, học viên</t>
+          <t>Người lao động (theo pháp luật về an toàn, vệ sinh lao động)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cơ Sở Khám Chữa Bệnh</t>
+          <t>Khám Lưu Động</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Người dân tự chi trả</t>
+          <t xml:space="preserve">Ngân sách thành phố hỗ trợ </t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Tự Thực hiện</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>Khám Theo Hợp Đồng</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>079099001234</t>
+          <t>087187000236</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NGUYEN VAN A</t>
+          <t>TRẦN NGỌC DUNG</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>01/01/1990</t>
+          <t>27/06/1987</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Nam</t>
+          <t>Nữ</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -3353,17 +4061,14 @@
           <t>Kinh</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
-          <t>0901234567</t>
+          <t>0989681925</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>123 Nguyen Trai</t>
+          <t>262/20 LẠC LONG QUÂN</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -3373,24 +4078,119 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
+          <t>Phường Bình Thới</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>GIÁO VIÊN MẦM NON</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 29/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Người lao động (theo pháp luật về an toàn, vệ sinh lao động)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Khám Lưu Động</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngân sách thành phố hỗ trợ </t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Khám Theo Hợp Đồng</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>079195031510</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>LE THI MAI</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>15/03/1995</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Kinh</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0989681920</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>45 Le Loi</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Thành Phố Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
           <t>Phường Hiệp Bình</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Nhân viên văn phòng</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Phòng khám đa khoa thuộc Công ty Cổ phần Bệnh viện Quốc tế European Wellness</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr">
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>GIÁO VIÊN MẦM NON</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 29/07/2026</t>
         </is>
       </c>
     </row>
@@ -3440,7 +4240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3853,6 +4653,57 @@
       <c r="C24" t="inlineStr">
         <is>
           <t>Lý do khám sức khỏe</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MaBanGhi</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>_output</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Script ghi — mã bản ghi trên web</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TrangThai</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>_output</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>THANH_CONG / TRUNG / LOI</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>GhiChu</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>_output</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Thông báo từ hệ thống</t>
         </is>
       </c>
     </row>

</xml_diff>